<commit_message>
Actualizacion modelos y app
</commit_message>
<xml_diff>
--- a/data/features_2.xlsx
+++ b/data/features_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PUT US\PUT-forecasting - modelo 3\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://televisaunivision-my.sharepoint.com/personal/gustavo_garduno_televisaunivision_com/Documents/2026/PUTS/PUT-forecasting - modelo 3  - Panel - Github/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD24997-AAFC-4F82-B61F-C80DF59B580C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="13_ncr:1_{CFD24997-AAFC-4F82-B61F-C80DF59B580C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{371AD36B-AFA2-4A37-B048-C914F8BDF3BA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{41D9290E-7B17-42E8-8E26-0530FE515D1F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{41D9290E-7B17-42E8-8E26-0530FE515D1F}"/>
   </bookViews>
   <sheets>
     <sheet name="dates" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,9 @@
     <sheet name="tnf" sheetId="3" r:id="rId4"/>
     <sheet name="descripción" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dates!$A$1:$O$103</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="238">
   <si>
     <t>newyear</t>
   </si>
@@ -732,12 +735,6 @@
     <t>Aún por disputarse</t>
   </si>
   <si>
-    <t>Jueves, 5 de junio de 2025 (Proyectado)</t>
-  </si>
-  <si>
-    <t>Domingo, 22 de junio de 2025 (Proyectado, si se requiere Juego 7)</t>
-  </si>
-  <si>
     <t>Pendiente</t>
   </si>
   <si>
@@ -793,6 +790,138 @@
   </si>
   <si>
     <t>**el resto es dicotómica</t>
+  </si>
+  <si>
+    <t>Oklahoma City Thunder vs. Indiana Pacers</t>
+  </si>
+  <si>
+    <t>Domingo, 22 de junio de 2025</t>
+  </si>
+  <si>
+    <t>Jueves, 1 de junio de 2027 (Proyectado)</t>
+  </si>
+  <si>
+    <t>Domingo, 20 de junio de 2027 (Proyectado, si se requiere Juego 7)</t>
+  </si>
+  <si>
+    <t>14 de septiembre de 2026</t>
+  </si>
+  <si>
+    <t>21 de septiembre de 2026</t>
+  </si>
+  <si>
+    <t>28 de septiembre de 2026</t>
+  </si>
+  <si>
+    <t>5 de octubre de 2026</t>
+  </si>
+  <si>
+    <t>12 de octubre de 2026</t>
+  </si>
+  <si>
+    <t>19 de octubre de 2026</t>
+  </si>
+  <si>
+    <t>26 de octubre de 2026</t>
+  </si>
+  <si>
+    <t>2 de noviembre de 2026</t>
+  </si>
+  <si>
+    <t>9 de noviembre de 2026</t>
+  </si>
+  <si>
+    <t>16 de noviembre de 2026</t>
+  </si>
+  <si>
+    <t>23 de noviembre de 2026</t>
+  </si>
+  <si>
+    <t>30 de noviembre de 2026</t>
+  </si>
+  <si>
+    <t>7 de diciembre de 2026</t>
+  </si>
+  <si>
+    <t>14 de diciembre de 2026</t>
+  </si>
+  <si>
+    <t>21 de diciembre de 2026</t>
+  </si>
+  <si>
+    <t>28 de diciembre de 2026</t>
+  </si>
+  <si>
+    <t>4 de enero de 2027</t>
+  </si>
+  <si>
+    <t>13 de septiembre de 2027</t>
+  </si>
+  <si>
+    <t>20 de septiembre de 2027</t>
+  </si>
+  <si>
+    <t>27 de septiembre de 2027</t>
+  </si>
+  <si>
+    <t>4 de octubre de 2027</t>
+  </si>
+  <si>
+    <t>11 de octubre de 2027</t>
+  </si>
+  <si>
+    <t>18 de octubre de 2027</t>
+  </si>
+  <si>
+    <t>25 de octubre de 2027</t>
+  </si>
+  <si>
+    <t>1 de noviembre de 2027</t>
+  </si>
+  <si>
+    <t>8 de noviembre de 2027</t>
+  </si>
+  <si>
+    <t>15 de noviembre de 2027</t>
+  </si>
+  <si>
+    <t>22 de noviembre de 2027</t>
+  </si>
+  <si>
+    <t>29 de noviembre de 2027</t>
+  </si>
+  <si>
+    <t>6 de diciembre de 2027</t>
+  </si>
+  <si>
+    <t>13 de diciembre de 2027</t>
+  </si>
+  <si>
+    <t>20 de diciembre de 2027</t>
+  </si>
+  <si>
+    <t>27 de diciembre de 2027</t>
+  </si>
+  <si>
+    <t>3 de enero de 2028</t>
+  </si>
+  <si>
+    <t>OKC</t>
+  </si>
+  <si>
+    <t>San Antonio Spurs vs. New York Knicks</t>
+  </si>
+  <si>
+    <t>NYK</t>
+  </si>
+  <si>
+    <t>Miercoles, 3 de junio de 2025</t>
+  </si>
+  <si>
+    <t>Sabado, 13 de junio de 2026</t>
+  </si>
+  <si>
+    <t>Jueves, 4 de junio de 2026</t>
   </si>
 </sst>
 </file>
@@ -802,7 +931,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -856,6 +985,19 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -932,7 +1074,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -958,6 +1100,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1295,54 +1447,63 @@
   <dimension ref="A1:O136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="3" width="10.90625" customWidth="1"/>
     <col min="4" max="4" width="13.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" customWidth="1"/>
+    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="10.90625" customWidth="1"/>
+    <col min="10" max="10" width="15" style="4" customWidth="1"/>
+    <col min="11" max="11" width="10.90625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="22.6328125" customWidth="1"/>
+    <col min="13" max="16" width="10.90625" customWidth="1"/>
+    <col min="17" max="17" width="33.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="18" t="s">
         <v>83</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>84</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -1373,12 +1534,11 @@
       <c r="I2" s="4">
         <v>44605</v>
       </c>
-      <c r="J2" s="4">
-        <f>H2-1</f>
-        <v>44815</v>
-      </c>
-      <c r="K2" s="4">
-        <v>45093</v>
+      <c r="J2" s="5">
+        <v>44563</v>
+      </c>
+      <c r="K2" s="5">
+        <v>46557</v>
       </c>
       <c r="L2" s="4">
         <v>45463</v>
@@ -1422,12 +1582,11 @@
       <c r="I3" s="4">
         <v>44969</v>
       </c>
-      <c r="J3" s="4">
-        <f t="shared" ref="J3:J17" si="1">H3-1</f>
-        <v>44822</v>
-      </c>
-      <c r="K3" s="4">
-        <v>45094</v>
+      <c r="J3" s="5">
+        <v>44601</v>
+      </c>
+      <c r="K3" s="5">
+        <v>46558</v>
       </c>
       <c r="L3" s="4">
         <v>45464</v>
@@ -1472,18 +1631,17 @@
       <c r="I4" s="4">
         <v>45333</v>
       </c>
-      <c r="J4" s="4">
-        <f t="shared" si="1"/>
-        <v>44829</v>
-      </c>
-      <c r="K4" s="4">
-        <v>45095</v>
+      <c r="J4" s="5">
+        <v>44577</v>
+      </c>
+      <c r="K4" s="5">
+        <v>46559</v>
       </c>
       <c r="L4" s="4">
         <v>45465</v>
       </c>
       <c r="M4" s="4">
-        <f t="shared" ref="M4:M18" si="2">M3+7</f>
+        <f t="shared" ref="M4:M18" si="1">M3+7</f>
         <v>44826</v>
       </c>
       <c r="N4" s="4">
@@ -1522,18 +1680,17 @@
       <c r="I5" s="4">
         <v>45697</v>
       </c>
-      <c r="J5" s="4">
-        <f t="shared" si="1"/>
-        <v>44836</v>
-      </c>
-      <c r="K5" s="4">
-        <v>45096</v>
+      <c r="J5" s="5">
+        <v>44584</v>
+      </c>
+      <c r="K5" s="5">
+        <v>46560</v>
       </c>
       <c r="L5" s="4">
         <v>45466</v>
       </c>
       <c r="M5" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44833</v>
       </c>
       <c r="N5" s="4">
@@ -1572,18 +1729,17 @@
       <c r="I6" s="5">
         <v>46061</v>
       </c>
-      <c r="J6" s="4">
-        <f t="shared" si="1"/>
-        <v>44843</v>
-      </c>
-      <c r="K6" s="4">
-        <v>45097</v>
+      <c r="J6" s="5">
+        <v>44591</v>
+      </c>
+      <c r="K6" s="5">
+        <v>46561</v>
       </c>
       <c r="L6" s="4">
         <v>45467</v>
       </c>
       <c r="M6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44840</v>
       </c>
       <c r="N6" s="4">
@@ -1623,17 +1779,17 @@
         <v>46432</v>
       </c>
       <c r="J7" s="4">
-        <f t="shared" si="1"/>
-        <v>44850</v>
-      </c>
-      <c r="K7" s="4">
-        <v>45098</v>
+        <f t="shared" ref="J7:J22" si="2">H2-1</f>
+        <v>44815</v>
+      </c>
+      <c r="K7" s="5">
+        <v>46562</v>
       </c>
       <c r="L7" s="4">
         <v>45468</v>
       </c>
       <c r="M7" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44847</v>
       </c>
       <c r="N7" s="4">
@@ -1656,17 +1812,17 @@
         <v>44858</v>
       </c>
       <c r="J8" s="4">
-        <f t="shared" si="1"/>
-        <v>44857</v>
-      </c>
-      <c r="K8" s="4">
-        <v>45099</v>
+        <f t="shared" si="2"/>
+        <v>44822</v>
+      </c>
+      <c r="K8" s="5">
+        <v>46563</v>
       </c>
       <c r="L8" s="4">
         <v>45469</v>
       </c>
       <c r="M8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44854</v>
       </c>
       <c r="N8" s="4">
@@ -1689,17 +1845,17 @@
         <v>44865</v>
       </c>
       <c r="J9" s="4">
-        <f t="shared" si="1"/>
-        <v>44864</v>
-      </c>
-      <c r="K9" s="4">
-        <v>45100</v>
+        <f t="shared" si="2"/>
+        <v>44829</v>
+      </c>
+      <c r="K9" s="5">
+        <v>46564</v>
       </c>
       <c r="L9" s="4">
         <v>45470</v>
       </c>
       <c r="M9" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44861</v>
       </c>
       <c r="N9" s="4">
@@ -1722,17 +1878,17 @@
         <v>44872</v>
       </c>
       <c r="J10" s="4">
-        <f t="shared" si="1"/>
-        <v>44871</v>
-      </c>
-      <c r="K10" s="4">
-        <v>45101</v>
+        <f t="shared" si="2"/>
+        <v>44836</v>
+      </c>
+      <c r="K10" s="5">
+        <v>46565</v>
       </c>
       <c r="L10" s="4">
         <v>45471</v>
       </c>
       <c r="M10" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44868</v>
       </c>
       <c r="N10" s="4">
@@ -1755,17 +1911,17 @@
         <v>44879</v>
       </c>
       <c r="J11" s="4">
-        <f t="shared" si="1"/>
-        <v>44878</v>
-      </c>
-      <c r="K11" s="4">
-        <v>45102</v>
+        <f t="shared" si="2"/>
+        <v>44843</v>
+      </c>
+      <c r="K11" s="5">
+        <v>46566</v>
       </c>
       <c r="L11" s="4">
         <v>45472</v>
       </c>
       <c r="M11" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44875</v>
       </c>
       <c r="N11" s="4">
@@ -1788,17 +1944,17 @@
         <v>44886</v>
       </c>
       <c r="J12" s="4">
-        <f t="shared" si="1"/>
-        <v>44885</v>
-      </c>
-      <c r="K12" s="4">
-        <v>45103</v>
+        <f t="shared" si="2"/>
+        <v>44850</v>
+      </c>
+      <c r="K12" s="5">
+        <v>46567</v>
       </c>
       <c r="L12" s="4">
         <v>45473</v>
       </c>
       <c r="M12" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44882</v>
       </c>
       <c r="N12" s="4">
@@ -1821,17 +1977,17 @@
         <v>44893</v>
       </c>
       <c r="J13" s="4">
-        <f t="shared" si="1"/>
-        <v>44892</v>
-      </c>
-      <c r="K13" s="4">
-        <v>45104</v>
+        <f t="shared" si="2"/>
+        <v>44857</v>
+      </c>
+      <c r="K13" s="5">
+        <v>46568</v>
       </c>
       <c r="L13" s="4">
         <v>45474</v>
       </c>
       <c r="M13" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44889</v>
       </c>
       <c r="N13" s="4">
@@ -1854,17 +2010,17 @@
         <v>44900</v>
       </c>
       <c r="J14" s="4">
-        <f t="shared" si="1"/>
-        <v>44899</v>
-      </c>
-      <c r="K14" s="4">
-        <v>45105</v>
+        <f t="shared" si="2"/>
+        <v>44864</v>
+      </c>
+      <c r="K14" s="5">
+        <v>46569</v>
       </c>
       <c r="L14" s="4">
         <v>45475</v>
       </c>
       <c r="M14" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44896</v>
       </c>
       <c r="N14" s="4">
@@ -1887,17 +2043,17 @@
         <v>44907</v>
       </c>
       <c r="J15" s="4">
-        <f t="shared" si="1"/>
-        <v>44906</v>
-      </c>
-      <c r="K15" s="4">
-        <v>45106</v>
+        <f t="shared" si="2"/>
+        <v>44871</v>
+      </c>
+      <c r="K15" s="5">
+        <v>46570</v>
       </c>
       <c r="L15" s="4">
         <v>45476</v>
       </c>
       <c r="M15" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44903</v>
       </c>
       <c r="N15" s="4">
@@ -1920,17 +2076,17 @@
         <v>44914</v>
       </c>
       <c r="J16" s="4">
-        <f t="shared" si="1"/>
-        <v>44913</v>
-      </c>
-      <c r="K16" s="4">
-        <v>45107</v>
+        <f t="shared" si="2"/>
+        <v>44878</v>
+      </c>
+      <c r="K16" s="5">
+        <v>46571</v>
       </c>
       <c r="L16" s="4">
         <v>45477</v>
       </c>
       <c r="M16" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44910</v>
       </c>
       <c r="N16" s="4">
@@ -1953,17 +2109,17 @@
         <v>44921</v>
       </c>
       <c r="J17" s="4">
-        <f t="shared" si="1"/>
-        <v>44920</v>
-      </c>
-      <c r="K17" s="4">
-        <v>45108</v>
+        <f t="shared" si="2"/>
+        <v>44885</v>
+      </c>
+      <c r="K17" s="5">
+        <v>46572</v>
       </c>
       <c r="L17" s="4">
         <v>45478</v>
       </c>
       <c r="M17" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44917</v>
       </c>
       <c r="N17" s="4">
@@ -1986,17 +2142,17 @@
         <v>44928</v>
       </c>
       <c r="J18" s="4">
-        <f>H19-1</f>
-        <v>45179</v>
-      </c>
-      <c r="K18" s="4">
-        <v>45109</v>
+        <f t="shared" si="2"/>
+        <v>44892</v>
+      </c>
+      <c r="K18" s="5">
+        <v>46573</v>
       </c>
       <c r="L18" s="4">
         <v>45479</v>
       </c>
       <c r="M18" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>44924</v>
       </c>
       <c r="N18" s="4">
@@ -2015,11 +2171,11 @@
         <v>45180</v>
       </c>
       <c r="J19" s="4">
-        <f t="shared" ref="J19:J34" si="3">H20-1</f>
-        <v>45186</v>
-      </c>
-      <c r="K19" s="4">
-        <v>45110</v>
+        <f t="shared" si="2"/>
+        <v>44899</v>
+      </c>
+      <c r="K19" s="5">
+        <v>46574</v>
       </c>
       <c r="L19" s="4">
         <v>45480</v>
@@ -2044,17 +2200,17 @@
         <v>45187</v>
       </c>
       <c r="J20" s="4">
-        <f t="shared" si="3"/>
-        <v>45193</v>
-      </c>
-      <c r="K20" s="4">
-        <v>45111</v>
+        <f t="shared" si="2"/>
+        <v>44906</v>
+      </c>
+      <c r="K20" s="5">
+        <v>46575</v>
       </c>
       <c r="L20" s="4">
         <v>45481</v>
       </c>
       <c r="M20" s="4">
-        <f t="shared" ref="M20:M32" si="4">M19+7</f>
+        <f t="shared" ref="M20:M32" si="3">M19+7</f>
         <v>45183</v>
       </c>
       <c r="N20" s="4">
@@ -2070,21 +2226,21 @@
         <v>44904</v>
       </c>
       <c r="H21" s="4">
-        <f t="shared" ref="H21:H34" si="5">H20+7</f>
+        <f t="shared" ref="H21:H34" si="4">H20+7</f>
         <v>45194</v>
       </c>
       <c r="J21" s="4">
-        <f t="shared" si="3"/>
-        <v>45200</v>
-      </c>
-      <c r="K21" s="4">
-        <v>45112</v>
+        <f t="shared" si="2"/>
+        <v>44913</v>
+      </c>
+      <c r="K21" s="5">
+        <v>46576</v>
       </c>
       <c r="L21" s="4">
         <v>45482</v>
       </c>
       <c r="M21" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45190</v>
       </c>
       <c r="N21" s="4">
@@ -2100,21 +2256,21 @@
         <v>44905</v>
       </c>
       <c r="H22" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45201</v>
       </c>
       <c r="J22" s="4">
-        <f t="shared" si="3"/>
-        <v>45207</v>
-      </c>
-      <c r="K22" s="4">
-        <v>45113</v>
+        <f t="shared" si="2"/>
+        <v>44920</v>
+      </c>
+      <c r="K22" s="5">
+        <v>46577</v>
       </c>
       <c r="L22" s="4">
         <v>45483</v>
       </c>
       <c r="M22" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45197</v>
       </c>
       <c r="N22" s="4">
@@ -2130,21 +2286,20 @@
         <v>44906</v>
       </c>
       <c r="H23" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45208</v>
       </c>
-      <c r="J23" s="4">
-        <f t="shared" si="3"/>
-        <v>45214</v>
-      </c>
-      <c r="K23" s="4">
-        <v>45114</v>
+      <c r="J23" s="5">
+        <v>44927</v>
+      </c>
+      <c r="K23" s="5">
+        <v>46578</v>
       </c>
       <c r="L23" s="4">
         <v>45484</v>
       </c>
       <c r="M23" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45204</v>
       </c>
       <c r="N23" s="4">
@@ -2160,25 +2315,24 @@
         <v>44907</v>
       </c>
       <c r="H24" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45215</v>
       </c>
-      <c r="J24" s="4">
-        <f t="shared" si="3"/>
-        <v>45221</v>
-      </c>
-      <c r="K24" s="4">
-        <v>45115</v>
+      <c r="J24" s="5">
+        <v>44934</v>
+      </c>
+      <c r="K24" s="5">
+        <v>46579</v>
       </c>
       <c r="L24" s="4">
         <v>45485</v>
       </c>
       <c r="M24" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45211</v>
       </c>
       <c r="N24" s="5">
-        <v>46177</v>
+        <v>46176</v>
       </c>
       <c r="O24" s="4">
         <v>45962</v>
@@ -2190,25 +2344,24 @@
         <v>44908</v>
       </c>
       <c r="H25" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45222</v>
       </c>
-      <c r="J25" s="4">
-        <f t="shared" si="3"/>
-        <v>45228</v>
-      </c>
-      <c r="K25" s="4">
-        <v>45116</v>
+      <c r="J25" s="5">
+        <v>44941</v>
+      </c>
+      <c r="K25" s="5">
+        <v>46580</v>
       </c>
       <c r="L25" s="4">
         <v>45486</v>
       </c>
       <c r="M25" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45218</v>
       </c>
       <c r="N25" s="5">
-        <v>46180</v>
+        <v>46178</v>
       </c>
       <c r="O25" s="5">
         <v>46318</v>
@@ -2220,25 +2373,24 @@
         <v>44909</v>
       </c>
       <c r="H26" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45229</v>
       </c>
-      <c r="J26" s="4">
-        <f t="shared" si="3"/>
-        <v>45235</v>
-      </c>
-      <c r="K26" s="4">
-        <v>45117</v>
+      <c r="J26" s="5">
+        <v>44948</v>
+      </c>
+      <c r="K26" s="5">
+        <v>46581</v>
       </c>
       <c r="L26" s="4">
         <v>45487</v>
       </c>
       <c r="M26" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45225</v>
       </c>
       <c r="N26" s="5">
-        <v>46183</v>
+        <v>46181</v>
       </c>
       <c r="O26" s="5">
         <v>46319</v>
@@ -2250,23 +2402,22 @@
         <v>44910</v>
       </c>
       <c r="H27" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45236</v>
       </c>
-      <c r="J27" s="4">
-        <f t="shared" si="3"/>
-        <v>45242</v>
-      </c>
-      <c r="K27" s="4">
-        <v>45118</v>
+      <c r="J27" s="5">
+        <v>44955</v>
+      </c>
+      <c r="K27" s="5">
+        <v>46582</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45232</v>
       </c>
       <c r="N27" s="5">
-        <v>46185</v>
+        <v>46183</v>
       </c>
       <c r="O27" s="5">
         <v>46321</v>
@@ -2278,23 +2429,23 @@
         <v>44911</v>
       </c>
       <c r="H28" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45243</v>
       </c>
       <c r="J28" s="4">
-        <f t="shared" si="3"/>
-        <v>45249</v>
-      </c>
-      <c r="K28" s="4">
-        <v>45119</v>
+        <f t="shared" ref="J28:J44" si="5">H19-1</f>
+        <v>45179</v>
+      </c>
+      <c r="K28" s="5">
+        <v>46583</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45239</v>
       </c>
       <c r="N28" s="5">
-        <v>46188</v>
+        <v>46186</v>
       </c>
       <c r="O28" s="5">
         <v>46322</v>
@@ -2306,23 +2457,23 @@
         <v>44912</v>
       </c>
       <c r="H29" s="4">
+        <f t="shared" si="4"/>
+        <v>45250</v>
+      </c>
+      <c r="J29" s="4">
         <f t="shared" si="5"/>
-        <v>45250</v>
-      </c>
-      <c r="J29" s="4">
-        <f t="shared" si="3"/>
-        <v>45256</v>
-      </c>
-      <c r="K29" s="4">
-        <v>45120</v>
+        <v>45186</v>
+      </c>
+      <c r="K29" s="5">
+        <v>46584</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45246</v>
       </c>
       <c r="N29" s="5">
-        <v>46191</v>
+        <v>46544</v>
       </c>
       <c r="O29" s="5">
         <v>46323</v>
@@ -2334,23 +2485,23 @@
         <v>44913</v>
       </c>
       <c r="H30" s="4">
+        <f t="shared" si="4"/>
+        <v>45257</v>
+      </c>
+      <c r="J30" s="4">
         <f t="shared" si="5"/>
-        <v>45257</v>
-      </c>
-      <c r="J30" s="4">
-        <f t="shared" si="3"/>
-        <v>45263</v>
-      </c>
-      <c r="K30" s="4">
-        <v>45121</v>
+        <v>45193</v>
+      </c>
+      <c r="K30" s="5">
+        <v>46585</v>
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45253</v>
       </c>
       <c r="N30" s="5">
-        <v>46541</v>
+        <v>46547</v>
       </c>
       <c r="O30" s="5">
         <v>46325</v>
@@ -2362,23 +2513,23 @@
         <v>46184</v>
       </c>
       <c r="H31" s="4">
+        <f t="shared" si="4"/>
+        <v>45264</v>
+      </c>
+      <c r="J31" s="4">
         <f t="shared" si="5"/>
-        <v>45264</v>
-      </c>
-      <c r="J31" s="4">
-        <f t="shared" si="3"/>
-        <v>45270</v>
-      </c>
-      <c r="K31" s="4">
-        <v>45122</v>
+        <v>45200</v>
+      </c>
+      <c r="K31" s="5">
+        <v>46586</v>
       </c>
       <c r="L31" s="1"/>
       <c r="M31" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45260</v>
       </c>
       <c r="N31" s="5">
-        <v>46544</v>
+        <v>46549</v>
       </c>
       <c r="O31" s="5">
         <v>46326</v>
@@ -2390,23 +2541,23 @@
         <v>46185</v>
       </c>
       <c r="H32" s="4">
+        <f t="shared" si="4"/>
+        <v>45271</v>
+      </c>
+      <c r="J32" s="4">
         <f t="shared" si="5"/>
-        <v>45271</v>
-      </c>
-      <c r="J32" s="4">
-        <f t="shared" si="3"/>
-        <v>45277</v>
-      </c>
-      <c r="K32" s="4">
-        <v>45123</v>
+        <v>45207</v>
+      </c>
+      <c r="K32" s="5">
+        <v>46587</v>
       </c>
       <c r="L32" s="1"/>
       <c r="M32" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>45267</v>
       </c>
       <c r="N32" s="5">
-        <v>46547</v>
+        <v>46552</v>
       </c>
       <c r="O32" s="5">
         <v>46682</v>
@@ -2418,15 +2569,15 @@
         <v>46186</v>
       </c>
       <c r="H33" s="4">
+        <f t="shared" si="4"/>
+        <v>45278</v>
+      </c>
+      <c r="J33" s="4">
         <f t="shared" si="5"/>
-        <v>45278</v>
-      </c>
-      <c r="J33" s="4">
-        <f t="shared" si="3"/>
-        <v>45284</v>
-      </c>
-      <c r="K33" s="5">
-        <v>46557</v>
+        <v>45214</v>
+      </c>
+      <c r="K33" s="4">
+        <v>45737</v>
       </c>
       <c r="L33" s="1"/>
       <c r="M33" s="4">
@@ -2434,7 +2585,7 @@
         <v>45274</v>
       </c>
       <c r="N33" s="5">
-        <v>46549</v>
+        <v>46555</v>
       </c>
       <c r="O33" s="5">
         <v>46683</v>
@@ -2446,15 +2597,15 @@
         <v>46187</v>
       </c>
       <c r="H34" s="4">
+        <f t="shared" si="4"/>
+        <v>45285</v>
+      </c>
+      <c r="J34" s="4">
         <f t="shared" si="5"/>
-        <v>45285</v>
-      </c>
-      <c r="J34" s="4">
-        <f t="shared" si="3"/>
-        <v>45289</v>
-      </c>
-      <c r="K34" s="5">
-        <v>46558</v>
+        <v>45221</v>
+      </c>
+      <c r="K34" s="4">
+        <v>45737</v>
       </c>
       <c r="L34" s="1"/>
       <c r="M34" s="4">
@@ -2462,7 +2613,7 @@
         <v>45281</v>
       </c>
       <c r="N34" s="5">
-        <v>46552</v>
+        <v>46559</v>
       </c>
       <c r="O34" s="5">
         <v>46685</v>
@@ -2477,20 +2628,17 @@
         <v>45290</v>
       </c>
       <c r="J35" s="4">
-        <f>H36-1</f>
-        <v>45543</v>
-      </c>
-      <c r="K35" s="5">
-        <v>46559</v>
+        <f t="shared" si="5"/>
+        <v>45228</v>
+      </c>
+      <c r="K35" s="4">
+        <v>45741</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="4">
         <f t="shared" ref="M35" si="6">M34+7</f>
         <v>45288</v>
       </c>
-      <c r="N35" s="5">
-        <v>46555</v>
-      </c>
       <c r="O35" s="5">
         <v>46686</v>
       </c>
@@ -2504,11 +2652,11 @@
         <v>45544</v>
       </c>
       <c r="J36" s="4">
-        <f t="shared" ref="J36:J51" si="7">H37-1</f>
-        <v>45550</v>
-      </c>
-      <c r="K36" s="5">
-        <v>46560</v>
+        <f t="shared" si="5"/>
+        <v>45235</v>
+      </c>
+      <c r="K36" s="4">
+        <v>45741</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="4">
@@ -2529,11 +2677,11 @@
         <v>45551</v>
       </c>
       <c r="J37" s="4">
-        <f t="shared" si="7"/>
-        <v>45557</v>
-      </c>
-      <c r="K37" s="5">
-        <v>46561</v>
+        <f t="shared" si="5"/>
+        <v>45242</v>
+      </c>
+      <c r="K37" s="4">
+        <v>45741</v>
       </c>
       <c r="L37" s="1"/>
       <c r="M37" s="4">
@@ -2550,19 +2698,19 @@
         <v>46191</v>
       </c>
       <c r="H38" s="4">
-        <f t="shared" ref="H38:H52" si="8">H37+7</f>
+        <f t="shared" ref="H38:H52" si="7">H37+7</f>
         <v>45558</v>
       </c>
       <c r="J38" s="4">
-        <f t="shared" si="7"/>
-        <v>45564</v>
-      </c>
-      <c r="K38" s="5">
-        <v>46562</v>
+        <f t="shared" si="5"/>
+        <v>45249</v>
+      </c>
+      <c r="K38" s="4">
+        <v>45741</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="4">
-        <f t="shared" ref="M38:M52" si="9">M37+7</f>
+        <f t="shared" ref="M38:M52" si="8">M37+7</f>
         <v>45554</v>
       </c>
       <c r="O38" s="5">
@@ -2575,19 +2723,19 @@
         <v>46192</v>
       </c>
       <c r="H39" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45565</v>
       </c>
       <c r="J39" s="4">
-        <f t="shared" si="7"/>
-        <v>45571</v>
-      </c>
-      <c r="K39" s="5">
-        <v>46563</v>
+        <f t="shared" si="5"/>
+        <v>45256</v>
+      </c>
+      <c r="K39" s="4">
+        <v>45741</v>
       </c>
       <c r="L39" s="1"/>
       <c r="M39" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45561</v>
       </c>
     </row>
@@ -2597,19 +2745,19 @@
         <v>46193</v>
       </c>
       <c r="H40" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45572</v>
       </c>
       <c r="J40" s="4">
-        <f t="shared" si="7"/>
-        <v>45578</v>
-      </c>
-      <c r="K40" s="5">
-        <v>46564</v>
+        <f t="shared" si="5"/>
+        <v>45263</v>
+      </c>
+      <c r="K40" s="4">
+        <v>45741</v>
       </c>
       <c r="L40" s="1"/>
       <c r="M40" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45568</v>
       </c>
     </row>
@@ -2619,19 +2767,19 @@
         <v>46194</v>
       </c>
       <c r="H41" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45579</v>
       </c>
       <c r="J41" s="4">
-        <f t="shared" si="7"/>
-        <v>45585</v>
-      </c>
-      <c r="K41" s="5">
-        <v>46565</v>
+        <f t="shared" si="5"/>
+        <v>45270</v>
+      </c>
+      <c r="K41" s="4">
+        <v>45741</v>
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45575</v>
       </c>
     </row>
@@ -2641,19 +2789,19 @@
         <v>46195</v>
       </c>
       <c r="H42" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45586</v>
       </c>
       <c r="J42" s="4">
-        <f t="shared" si="7"/>
-        <v>45592</v>
-      </c>
-      <c r="K42" s="5">
-        <v>46566</v>
+        <f t="shared" si="5"/>
+        <v>45277</v>
+      </c>
+      <c r="K42" s="4">
+        <v>45822</v>
       </c>
       <c r="L42" s="1"/>
       <c r="M42" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45582</v>
       </c>
     </row>
@@ -2663,15 +2811,15 @@
         <v>46196</v>
       </c>
       <c r="H43" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45593</v>
       </c>
       <c r="J43" s="4">
-        <f t="shared" si="7"/>
-        <v>45599</v>
-      </c>
-      <c r="K43" s="5">
-        <v>46567</v>
+        <f t="shared" si="5"/>
+        <v>45284</v>
+      </c>
+      <c r="K43" s="4">
+        <v>45823</v>
       </c>
       <c r="L43" s="1"/>
       <c r="M43" s="4">
@@ -2685,19 +2833,19 @@
         <v>46197</v>
       </c>
       <c r="H44" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45600</v>
       </c>
       <c r="J44" s="4">
-        <f t="shared" si="7"/>
-        <v>45606</v>
-      </c>
-      <c r="K44" s="5">
-        <v>46568</v>
+        <f t="shared" si="5"/>
+        <v>45289</v>
+      </c>
+      <c r="K44" s="4">
+        <v>45823</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45596</v>
       </c>
     </row>
@@ -2707,19 +2855,18 @@
         <v>46198</v>
       </c>
       <c r="H45" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45607</v>
       </c>
-      <c r="J45" s="4">
-        <f t="shared" si="7"/>
-        <v>45613</v>
-      </c>
-      <c r="K45" s="5">
-        <v>46569</v>
+      <c r="J45" s="5">
+        <v>45298</v>
+      </c>
+      <c r="K45" s="4">
+        <v>45823</v>
       </c>
       <c r="L45" s="1"/>
       <c r="M45" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45603</v>
       </c>
     </row>
@@ -2732,16 +2879,15 @@
         <f>H45+7</f>
         <v>45614</v>
       </c>
-      <c r="J46" s="4">
-        <f>H47-1</f>
-        <v>45620</v>
-      </c>
-      <c r="K46" s="5">
-        <v>46570</v>
+      <c r="J46" s="5">
+        <v>45305</v>
+      </c>
+      <c r="K46" s="4">
+        <v>45824</v>
       </c>
       <c r="L46" s="1"/>
       <c r="M46" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45610</v>
       </c>
     </row>
@@ -2751,18 +2897,17 @@
         <v>46200</v>
       </c>
       <c r="H47" s="4">
+        <f t="shared" si="7"/>
+        <v>45621</v>
+      </c>
+      <c r="J47" s="5">
+        <v>45312</v>
+      </c>
+      <c r="K47" s="4">
+        <v>45824</v>
+      </c>
+      <c r="M47" s="4">
         <f t="shared" si="8"/>
-        <v>45621</v>
-      </c>
-      <c r="J47" s="4">
-        <f t="shared" si="7"/>
-        <v>45627</v>
-      </c>
-      <c r="K47" s="5">
-        <v>46571</v>
-      </c>
-      <c r="M47" s="4">
-        <f t="shared" si="9"/>
         <v>45617</v>
       </c>
     </row>
@@ -2772,15 +2917,14 @@
         <v>46201</v>
       </c>
       <c r="H48" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>45628</v>
       </c>
-      <c r="J48" s="4">
-        <f t="shared" si="7"/>
-        <v>45634</v>
-      </c>
-      <c r="K48" s="5">
-        <v>46572</v>
+      <c r="J48" s="5">
+        <v>45319</v>
+      </c>
+      <c r="K48" s="4">
+        <v>45825</v>
       </c>
       <c r="M48" s="4">
         <f>M47+7</f>
@@ -2793,18 +2937,18 @@
         <v>46202</v>
       </c>
       <c r="H49" s="4">
+        <f t="shared" si="7"/>
+        <v>45635</v>
+      </c>
+      <c r="J49" s="4">
+        <f t="shared" ref="J49:J65" si="9">H36-1</f>
+        <v>45543</v>
+      </c>
+      <c r="K49" s="4">
+        <v>45825</v>
+      </c>
+      <c r="M49" s="4">
         <f t="shared" si="8"/>
-        <v>45635</v>
-      </c>
-      <c r="J49" s="4">
-        <f t="shared" si="7"/>
-        <v>45641</v>
-      </c>
-      <c r="K49" s="5">
-        <v>46573</v>
-      </c>
-      <c r="M49" s="4">
-        <f t="shared" si="9"/>
         <v>45631</v>
       </c>
     </row>
@@ -2814,18 +2958,18 @@
         <v>46203</v>
       </c>
       <c r="H50" s="4">
+        <f t="shared" si="7"/>
+        <v>45642</v>
+      </c>
+      <c r="J50" s="4">
+        <f t="shared" si="9"/>
+        <v>45550</v>
+      </c>
+      <c r="K50" s="4">
+        <v>45826</v>
+      </c>
+      <c r="M50" s="4">
         <f t="shared" si="8"/>
-        <v>45642</v>
-      </c>
-      <c r="J50" s="4">
-        <f t="shared" si="7"/>
-        <v>45648</v>
-      </c>
-      <c r="K50" s="5">
-        <v>46574</v>
-      </c>
-      <c r="M50" s="4">
-        <f t="shared" si="9"/>
         <v>45638</v>
       </c>
     </row>
@@ -2839,14 +2983,14 @@
         <v>45649</v>
       </c>
       <c r="J51" s="4">
-        <f t="shared" si="7"/>
-        <v>45655</v>
-      </c>
-      <c r="K51" s="5">
-        <v>46575</v>
+        <f t="shared" si="9"/>
+        <v>45557</v>
+      </c>
+      <c r="K51" s="4">
+        <v>45826</v>
       </c>
       <c r="M51" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>45645</v>
       </c>
     </row>
@@ -2856,18 +3000,18 @@
         <v>46205</v>
       </c>
       <c r="H52" s="4">
+        <f t="shared" si="7"/>
+        <v>45656</v>
+      </c>
+      <c r="J52" s="4">
+        <f t="shared" si="9"/>
+        <v>45564</v>
+      </c>
+      <c r="K52" s="4">
+        <v>45827</v>
+      </c>
+      <c r="M52" s="4">
         <f t="shared" si="8"/>
-        <v>45656</v>
-      </c>
-      <c r="J52" s="4">
-        <f>H53-1</f>
-        <v>45907</v>
-      </c>
-      <c r="K52" s="5">
-        <v>46576</v>
-      </c>
-      <c r="M52" s="4">
-        <f t="shared" si="9"/>
         <v>45652</v>
       </c>
     </row>
@@ -2880,11 +3024,11 @@
         <v>45908</v>
       </c>
       <c r="J53" s="4">
-        <f t="shared" ref="J53:J67" si="10">H54-1</f>
-        <v>45914</v>
-      </c>
-      <c r="K53" s="5">
-        <v>46577</v>
+        <f t="shared" si="9"/>
+        <v>45571</v>
+      </c>
+      <c r="K53" s="4">
+        <v>45827</v>
       </c>
       <c r="M53" s="4">
         <v>45904</v>
@@ -2900,11 +3044,11 @@
         <v>45915</v>
       </c>
       <c r="J54" s="4">
-        <f t="shared" si="10"/>
-        <v>45921</v>
-      </c>
-      <c r="K54" s="5">
-        <v>46578</v>
+        <f t="shared" si="9"/>
+        <v>45578</v>
+      </c>
+      <c r="K54" s="4">
+        <v>45828</v>
       </c>
       <c r="M54" s="4">
         <f>M53+7</f>
@@ -2917,18 +3061,18 @@
         <v>46208</v>
       </c>
       <c r="H55" s="4">
-        <f t="shared" ref="H55:H69" si="11">H54+7</f>
+        <f t="shared" ref="H55:H69" si="10">H54+7</f>
         <v>45922</v>
       </c>
       <c r="J55" s="4">
-        <f t="shared" si="10"/>
-        <v>45928</v>
-      </c>
-      <c r="K55" s="5">
-        <v>46579</v>
+        <f t="shared" si="9"/>
+        <v>45585</v>
+      </c>
+      <c r="K55" s="4">
+        <v>45828</v>
       </c>
       <c r="M55" s="4">
-        <f t="shared" ref="M55:M69" si="12">M54+7</f>
+        <f t="shared" ref="M55:M69" si="11">M54+7</f>
         <v>45918</v>
       </c>
     </row>
@@ -2938,18 +3082,18 @@
         <v>46209</v>
       </c>
       <c r="H56" s="4">
+        <f t="shared" si="10"/>
+        <v>45929</v>
+      </c>
+      <c r="J56" s="4">
+        <f t="shared" si="9"/>
+        <v>45592</v>
+      </c>
+      <c r="K56" s="4">
+        <v>45829</v>
+      </c>
+      <c r="M56" s="4">
         <f t="shared" si="11"/>
-        <v>45929</v>
-      </c>
-      <c r="J56" s="4">
-        <f t="shared" si="10"/>
-        <v>45935</v>
-      </c>
-      <c r="K56" s="5">
-        <v>46580</v>
-      </c>
-      <c r="M56" s="4">
-        <f t="shared" si="12"/>
         <v>45925</v>
       </c>
     </row>
@@ -2959,18 +3103,18 @@
         <v>46210</v>
       </c>
       <c r="H57" s="4">
+        <f t="shared" si="10"/>
+        <v>45936</v>
+      </c>
+      <c r="J57" s="4">
+        <f t="shared" si="9"/>
+        <v>45599</v>
+      </c>
+      <c r="K57" s="4">
+        <v>45829</v>
+      </c>
+      <c r="M57" s="4">
         <f t="shared" si="11"/>
-        <v>45936</v>
-      </c>
-      <c r="J57" s="4">
-        <f t="shared" si="10"/>
-        <v>45942</v>
-      </c>
-      <c r="K57" s="5">
-        <v>46581</v>
-      </c>
-      <c r="M57" s="4">
-        <f t="shared" si="12"/>
         <v>45932</v>
       </c>
     </row>
@@ -2980,18 +3124,18 @@
         <v>46211</v>
       </c>
       <c r="H58" s="4">
+        <f t="shared" si="10"/>
+        <v>45943</v>
+      </c>
+      <c r="J58" s="4">
+        <f t="shared" si="9"/>
+        <v>45606</v>
+      </c>
+      <c r="K58" s="4">
+        <v>45830</v>
+      </c>
+      <c r="M58" s="4">
         <f t="shared" si="11"/>
-        <v>45943</v>
-      </c>
-      <c r="J58" s="4">
-        <f t="shared" si="10"/>
-        <v>45949</v>
-      </c>
-      <c r="K58" s="5">
-        <v>46582</v>
-      </c>
-      <c r="M58" s="4">
-        <f t="shared" si="12"/>
         <v>45939</v>
       </c>
     </row>
@@ -3001,18 +3145,18 @@
         <v>46212</v>
       </c>
       <c r="H59" s="4">
+        <f t="shared" si="10"/>
+        <v>45950</v>
+      </c>
+      <c r="J59" s="4">
+        <f t="shared" si="9"/>
+        <v>45613</v>
+      </c>
+      <c r="K59" s="4">
+        <v>45830</v>
+      </c>
+      <c r="M59" s="4">
         <f t="shared" si="11"/>
-        <v>45950</v>
-      </c>
-      <c r="J59" s="4">
-        <f t="shared" si="10"/>
-        <v>45956</v>
-      </c>
-      <c r="K59" s="5">
-        <v>46583</v>
-      </c>
-      <c r="M59" s="4">
-        <f t="shared" si="12"/>
         <v>45946</v>
       </c>
     </row>
@@ -3022,18 +3166,18 @@
         <v>46213</v>
       </c>
       <c r="H60" s="4">
+        <f t="shared" si="10"/>
+        <v>45957</v>
+      </c>
+      <c r="J60" s="4">
+        <f t="shared" si="9"/>
+        <v>45620</v>
+      </c>
+      <c r="K60" s="4">
+        <v>45830</v>
+      </c>
+      <c r="M60" s="4">
         <f t="shared" si="11"/>
-        <v>45957</v>
-      </c>
-      <c r="J60" s="5">
-        <f t="shared" si="10"/>
-        <v>45963</v>
-      </c>
-      <c r="K60" s="5">
-        <v>46584</v>
-      </c>
-      <c r="M60" s="4">
-        <f t="shared" si="12"/>
         <v>45953</v>
       </c>
     </row>
@@ -3043,18 +3187,18 @@
         <v>46214</v>
       </c>
       <c r="H61" s="5">
+        <f t="shared" si="10"/>
+        <v>45964</v>
+      </c>
+      <c r="J61" s="4">
+        <f t="shared" si="9"/>
+        <v>45627</v>
+      </c>
+      <c r="K61" s="4">
+        <v>45830</v>
+      </c>
+      <c r="M61" s="4">
         <f t="shared" si="11"/>
-        <v>45964</v>
-      </c>
-      <c r="J61" s="5">
-        <f t="shared" si="10"/>
-        <v>45970</v>
-      </c>
-      <c r="K61" s="5">
-        <v>46585</v>
-      </c>
-      <c r="M61" s="4">
-        <f t="shared" si="12"/>
         <v>45960</v>
       </c>
     </row>
@@ -3064,18 +3208,18 @@
         <v>46215</v>
       </c>
       <c r="H62" s="5">
+        <f t="shared" si="10"/>
+        <v>45971</v>
+      </c>
+      <c r="J62" s="4">
+        <f t="shared" si="9"/>
+        <v>45634</v>
+      </c>
+      <c r="K62" s="4">
+        <v>45832</v>
+      </c>
+      <c r="M62" s="4">
         <f t="shared" si="11"/>
-        <v>45971</v>
-      </c>
-      <c r="J62" s="5">
-        <f t="shared" si="10"/>
-        <v>45977</v>
-      </c>
-      <c r="K62" s="5">
-        <v>46586</v>
-      </c>
-      <c r="M62" s="4">
-        <f t="shared" si="12"/>
         <v>45967</v>
       </c>
     </row>
@@ -3085,18 +3229,18 @@
         <v>46216</v>
       </c>
       <c r="H63" s="5">
+        <f t="shared" si="10"/>
+        <v>45978</v>
+      </c>
+      <c r="J63" s="4">
+        <f t="shared" si="9"/>
+        <v>45641</v>
+      </c>
+      <c r="K63" s="4">
+        <v>45832</v>
+      </c>
+      <c r="M63" s="4">
         <f t="shared" si="11"/>
-        <v>45978</v>
-      </c>
-      <c r="J63" s="5">
-        <f t="shared" si="10"/>
-        <v>45984</v>
-      </c>
-      <c r="K63" s="5">
-        <v>46587</v>
-      </c>
-      <c r="M63" s="4">
-        <f t="shared" si="12"/>
         <v>45974</v>
       </c>
     </row>
@@ -3106,15 +3250,18 @@
         <v>46217</v>
       </c>
       <c r="H64" s="5">
+        <f t="shared" si="10"/>
+        <v>45985</v>
+      </c>
+      <c r="J64" s="4">
+        <f t="shared" si="9"/>
+        <v>45648</v>
+      </c>
+      <c r="K64" s="4">
+        <v>45832</v>
+      </c>
+      <c r="M64" s="4">
         <f t="shared" si="11"/>
-        <v>45985</v>
-      </c>
-      <c r="J64" s="5">
-        <f t="shared" si="10"/>
-        <v>45991</v>
-      </c>
-      <c r="M64" s="4">
-        <f t="shared" si="12"/>
         <v>45981</v>
       </c>
     </row>
@@ -3124,15 +3271,18 @@
         <v>46218</v>
       </c>
       <c r="H65" s="5">
+        <f t="shared" si="10"/>
+        <v>45992</v>
+      </c>
+      <c r="J65" s="4">
+        <f t="shared" si="9"/>
+        <v>45655</v>
+      </c>
+      <c r="K65" s="4">
+        <v>45832</v>
+      </c>
+      <c r="M65" s="4">
         <f t="shared" si="11"/>
-        <v>45992</v>
-      </c>
-      <c r="J65" s="5">
-        <f t="shared" si="10"/>
-        <v>45998</v>
-      </c>
-      <c r="M65" s="4">
-        <f t="shared" si="12"/>
         <v>45988</v>
       </c>
     </row>
@@ -3142,15 +3292,17 @@
         <v>46219</v>
       </c>
       <c r="H66" s="5">
+        <f t="shared" si="10"/>
+        <v>45999</v>
+      </c>
+      <c r="J66" s="5">
+        <v>45662</v>
+      </c>
+      <c r="K66" s="4">
+        <v>45836</v>
+      </c>
+      <c r="M66" s="4">
         <f t="shared" si="11"/>
-        <v>45999</v>
-      </c>
-      <c r="J66" s="5">
-        <f t="shared" si="10"/>
-        <v>46005</v>
-      </c>
-      <c r="M66" s="4">
-        <f t="shared" si="12"/>
         <v>45995</v>
       </c>
     </row>
@@ -3160,15 +3312,17 @@
         <v>46220</v>
       </c>
       <c r="H67" s="5">
+        <f t="shared" si="10"/>
+        <v>46006</v>
+      </c>
+      <c r="J67" s="5">
+        <v>45669</v>
+      </c>
+      <c r="K67" s="4">
+        <v>45836</v>
+      </c>
+      <c r="M67" s="4">
         <f t="shared" si="11"/>
-        <v>46006</v>
-      </c>
-      <c r="J67" s="5">
-        <f t="shared" si="10"/>
-        <v>46012</v>
-      </c>
-      <c r="M67" s="4">
-        <f t="shared" si="12"/>
         <v>46002</v>
       </c>
     </row>
@@ -3178,15 +3332,17 @@
         <v>46221</v>
       </c>
       <c r="H68" s="5">
+        <f t="shared" si="10"/>
+        <v>46013</v>
+      </c>
+      <c r="J68" s="5">
+        <v>45676</v>
+      </c>
+      <c r="K68" s="4">
+        <v>45837</v>
+      </c>
+      <c r="M68" s="4">
         <f t="shared" si="11"/>
-        <v>46013</v>
-      </c>
-      <c r="J68" s="5">
-        <f t="shared" ref="J68:J103" si="13">H69-1</f>
-        <v>46019</v>
-      </c>
-      <c r="M68" s="4">
-        <f t="shared" si="12"/>
         <v>46009</v>
       </c>
     </row>
@@ -3196,26 +3352,31 @@
         <v>46222</v>
       </c>
       <c r="H69" s="5">
+        <f t="shared" si="10"/>
+        <v>46020</v>
+      </c>
+      <c r="J69" s="5">
+        <v>45683</v>
+      </c>
+      <c r="K69" s="4">
+        <v>45837</v>
+      </c>
+      <c r="M69" s="4">
         <f t="shared" si="11"/>
-        <v>46020</v>
-      </c>
-      <c r="J69" s="5">
-        <f t="shared" si="13"/>
-        <v>46271</v>
-      </c>
-      <c r="M69" s="4">
-        <f t="shared" si="12"/>
         <v>46016</v>
       </c>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B70" s="1"/>
       <c r="H70" s="5">
-        <v>46272</v>
-      </c>
-      <c r="J70" s="5">
-        <f t="shared" si="13"/>
-        <v>46278</v>
+        <v>46279</v>
+      </c>
+      <c r="J70" s="4">
+        <f t="shared" ref="J70:J86" si="12">H53-1</f>
+        <v>45907</v>
+      </c>
+      <c r="K70" s="4">
+        <v>45840</v>
       </c>
       <c r="M70" s="5">
         <v>46275</v>
@@ -3224,11 +3385,15 @@
     <row r="71" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B71" s="1"/>
       <c r="H71" s="5">
-        <v>46279</v>
-      </c>
-      <c r="J71" s="5">
-        <f t="shared" si="13"/>
-        <v>46285</v>
+        <f t="shared" ref="H71:H86" si="13">H70+7</f>
+        <v>46286</v>
+      </c>
+      <c r="J71" s="4">
+        <f t="shared" si="12"/>
+        <v>45914</v>
+      </c>
+      <c r="K71" s="4">
+        <v>45840</v>
       </c>
       <c r="M71" s="5">
         <f>M70+7</f>
@@ -3238,12 +3403,15 @@
     <row r="72" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B72" s="1"/>
       <c r="H72" s="5">
-        <f>H71+7</f>
-        <v>46286</v>
-      </c>
-      <c r="J72" s="5">
         <f t="shared" si="13"/>
-        <v>46292</v>
+        <v>46293</v>
+      </c>
+      <c r="J72" s="4">
+        <f t="shared" si="12"/>
+        <v>45921</v>
+      </c>
+      <c r="K72" s="4">
+        <v>45844</v>
       </c>
       <c r="M72" s="5">
         <f>M71+7</f>
@@ -3253,222 +3421,265 @@
     <row r="73" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B73" s="1"/>
       <c r="H73" s="5">
-        <f t="shared" ref="H73:H87" si="14">H72+7</f>
-        <v>46293</v>
-      </c>
-      <c r="J73" s="5">
         <f t="shared" si="13"/>
-        <v>46299</v>
+        <v>46300</v>
+      </c>
+      <c r="J73" s="4">
+        <f t="shared" si="12"/>
+        <v>45928</v>
+      </c>
+      <c r="K73" s="4">
+        <v>45093</v>
       </c>
       <c r="M73" s="5">
-        <f t="shared" ref="M73:M86" si="15">M72+7</f>
+        <f t="shared" ref="M73:M86" si="14">M72+7</f>
         <v>46296</v>
       </c>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B74" s="1"/>
       <c r="H74" s="5">
+        <f t="shared" si="13"/>
+        <v>46307</v>
+      </c>
+      <c r="J74" s="4">
+        <f t="shared" si="12"/>
+        <v>45935</v>
+      </c>
+      <c r="K74" s="4">
+        <v>45094</v>
+      </c>
+      <c r="M74" s="5">
         <f t="shared" si="14"/>
-        <v>46300</v>
-      </c>
-      <c r="J74" s="5">
-        <f t="shared" si="13"/>
-        <v>46306</v>
-      </c>
-      <c r="M74" s="5">
-        <f t="shared" si="15"/>
         <v>46303</v>
       </c>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B75" s="1"/>
       <c r="H75" s="5">
+        <f t="shared" si="13"/>
+        <v>46314</v>
+      </c>
+      <c r="J75" s="4">
+        <f t="shared" si="12"/>
+        <v>45942</v>
+      </c>
+      <c r="K75" s="4">
+        <v>45097</v>
+      </c>
+      <c r="M75" s="5">
         <f t="shared" si="14"/>
-        <v>46307</v>
-      </c>
-      <c r="J75" s="5">
-        <f t="shared" si="13"/>
-        <v>46313</v>
-      </c>
-      <c r="M75" s="5">
-        <f t="shared" si="15"/>
         <v>46310</v>
       </c>
     </row>
     <row r="76" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B76" s="1"/>
       <c r="H76" s="5">
+        <f t="shared" si="13"/>
+        <v>46321</v>
+      </c>
+      <c r="J76" s="4">
+        <f t="shared" si="12"/>
+        <v>45949</v>
+      </c>
+      <c r="K76" s="4">
+        <v>45101</v>
+      </c>
+      <c r="M76" s="5">
         <f t="shared" si="14"/>
-        <v>46314</v>
-      </c>
-      <c r="J76" s="5">
-        <f t="shared" si="13"/>
-        <v>46320</v>
-      </c>
-      <c r="M76" s="5">
-        <f t="shared" si="15"/>
         <v>46317</v>
       </c>
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B77" s="1"/>
       <c r="H77" s="5">
+        <f t="shared" si="13"/>
+        <v>46328</v>
+      </c>
+      <c r="J77" s="4">
+        <f t="shared" si="12"/>
+        <v>45956</v>
+      </c>
+      <c r="K77" s="4">
+        <v>45102</v>
+      </c>
+      <c r="M77" s="5">
         <f t="shared" si="14"/>
-        <v>46321</v>
-      </c>
-      <c r="J77" s="5">
-        <f t="shared" si="13"/>
-        <v>46327</v>
-      </c>
-      <c r="M77" s="5">
-        <f t="shared" si="15"/>
         <v>46324</v>
       </c>
     </row>
     <row r="78" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B78" s="1"/>
       <c r="H78" s="5">
+        <f t="shared" si="13"/>
+        <v>46335</v>
+      </c>
+      <c r="J78" s="5">
+        <f t="shared" si="12"/>
+        <v>45963</v>
+      </c>
+      <c r="K78" s="4">
+        <v>45103</v>
+      </c>
+      <c r="M78" s="5">
         <f t="shared" si="14"/>
-        <v>46328</v>
-      </c>
-      <c r="J78" s="5">
-        <f t="shared" si="13"/>
-        <v>46334</v>
-      </c>
-      <c r="M78" s="5">
-        <f t="shared" si="15"/>
         <v>46331</v>
       </c>
     </row>
     <row r="79" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B79" s="1"/>
       <c r="H79" s="5">
+        <f t="shared" si="13"/>
+        <v>46342</v>
+      </c>
+      <c r="J79" s="5">
+        <f t="shared" si="12"/>
+        <v>45970</v>
+      </c>
+      <c r="K79" s="4">
+        <v>45104</v>
+      </c>
+      <c r="M79" s="5">
         <f t="shared" si="14"/>
-        <v>46335</v>
-      </c>
-      <c r="J79" s="5">
-        <f t="shared" si="13"/>
-        <v>46341</v>
-      </c>
-      <c r="M79" s="5">
-        <f t="shared" si="15"/>
         <v>46338</v>
       </c>
     </row>
     <row r="80" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B80" s="1"/>
       <c r="H80" s="5">
+        <f t="shared" si="13"/>
+        <v>46349</v>
+      </c>
+      <c r="J80" s="5">
+        <f t="shared" si="12"/>
+        <v>45977</v>
+      </c>
+      <c r="K80" s="4">
+        <v>45105</v>
+      </c>
+      <c r="M80" s="5">
         <f t="shared" si="14"/>
-        <v>46342</v>
-      </c>
-      <c r="J80" s="5">
-        <f t="shared" si="13"/>
-        <v>46348</v>
-      </c>
-      <c r="M80" s="5">
-        <f t="shared" si="15"/>
         <v>46345</v>
       </c>
     </row>
     <row r="81" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B81" s="1"/>
       <c r="H81" s="5">
+        <f t="shared" si="13"/>
+        <v>46356</v>
+      </c>
+      <c r="J81" s="5">
+        <f t="shared" si="12"/>
+        <v>45984</v>
+      </c>
+      <c r="K81" s="4">
+        <v>45106</v>
+      </c>
+      <c r="M81" s="5">
         <f t="shared" si="14"/>
-        <v>46349</v>
-      </c>
-      <c r="J81" s="5">
-        <f t="shared" si="13"/>
-        <v>46355</v>
-      </c>
-      <c r="M81" s="5">
-        <f t="shared" si="15"/>
         <v>46352</v>
       </c>
     </row>
     <row r="82" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B82" s="1"/>
       <c r="H82" s="5">
+        <f t="shared" si="13"/>
+        <v>46363</v>
+      </c>
+      <c r="J82" s="5">
+        <f t="shared" si="12"/>
+        <v>45991</v>
+      </c>
+      <c r="K82" s="4">
+        <v>45107</v>
+      </c>
+      <c r="M82" s="5">
         <f t="shared" si="14"/>
-        <v>46356</v>
-      </c>
-      <c r="J82" s="5">
-        <f t="shared" si="13"/>
-        <v>46362</v>
-      </c>
-      <c r="M82" s="5">
-        <f t="shared" si="15"/>
         <v>46359</v>
       </c>
     </row>
     <row r="83" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B83" s="1"/>
       <c r="H83" s="5">
+        <f t="shared" si="13"/>
+        <v>46370</v>
+      </c>
+      <c r="J83" s="5">
+        <f t="shared" si="12"/>
+        <v>45998</v>
+      </c>
+      <c r="K83" s="4">
+        <v>45108</v>
+      </c>
+      <c r="M83" s="5">
         <f t="shared" si="14"/>
-        <v>46363</v>
-      </c>
-      <c r="J83" s="5">
-        <f t="shared" si="13"/>
-        <v>46369</v>
-      </c>
-      <c r="M83" s="5">
-        <f t="shared" si="15"/>
         <v>46366</v>
       </c>
     </row>
     <row r="84" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B84" s="1"/>
       <c r="H84" s="5">
+        <f t="shared" si="13"/>
+        <v>46377</v>
+      </c>
+      <c r="J84" s="5">
+        <f t="shared" si="12"/>
+        <v>46005</v>
+      </c>
+      <c r="K84" s="4">
+        <v>45109</v>
+      </c>
+      <c r="M84" s="5">
         <f t="shared" si="14"/>
-        <v>46370</v>
-      </c>
-      <c r="J84" s="5">
-        <f t="shared" si="13"/>
-        <v>46376</v>
-      </c>
-      <c r="M84" s="5">
-        <f t="shared" si="15"/>
         <v>46373</v>
       </c>
     </row>
     <row r="85" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B85" s="1"/>
       <c r="H85" s="5">
+        <f t="shared" si="13"/>
+        <v>46384</v>
+      </c>
+      <c r="J85" s="5">
+        <f t="shared" si="12"/>
+        <v>46012</v>
+      </c>
+      <c r="K85" s="4">
+        <v>45111</v>
+      </c>
+      <c r="M85" s="5">
         <f t="shared" si="14"/>
-        <v>46377</v>
-      </c>
-      <c r="J85" s="5">
-        <f t="shared" si="13"/>
-        <v>46383</v>
-      </c>
-      <c r="M85" s="5">
-        <f t="shared" si="15"/>
         <v>46380</v>
       </c>
     </row>
     <row r="86" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B86" s="1"/>
       <c r="H86" s="5">
+        <f t="shared" si="13"/>
+        <v>46391</v>
+      </c>
+      <c r="J86" s="5">
+        <f t="shared" si="12"/>
+        <v>46019</v>
+      </c>
+      <c r="K86" s="4">
+        <v>45115</v>
+      </c>
+      <c r="M86" s="5">
         <f t="shared" si="14"/>
-        <v>46384</v>
-      </c>
-      <c r="J86" s="5">
-        <f t="shared" si="13"/>
-        <v>46390</v>
-      </c>
-      <c r="M86" s="5">
-        <f t="shared" si="15"/>
         <v>46387</v>
       </c>
     </row>
     <row r="87" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B87" s="1"/>
       <c r="H87" s="5">
-        <f t="shared" si="14"/>
-        <v>46391</v>
-      </c>
-      <c r="J87" s="5">
-        <f t="shared" si="13"/>
-        <v>46642</v>
+        <v>46643</v>
+      </c>
+      <c r="J87" s="4">
+        <v>46026</v>
+      </c>
+      <c r="K87" s="4">
+        <v>45116</v>
       </c>
       <c r="M87" s="5">
         <v>46639</v>
@@ -3477,11 +3688,14 @@
     <row r="88" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B88" s="1"/>
       <c r="H88" s="5">
-        <v>46643</v>
-      </c>
-      <c r="J88" s="5">
-        <f t="shared" si="13"/>
-        <v>46649</v>
+        <f>H87+7</f>
+        <v>46650</v>
+      </c>
+      <c r="J88" s="4">
+        <v>46033</v>
+      </c>
+      <c r="K88" s="4">
+        <v>45119</v>
       </c>
       <c r="M88" s="5">
         <f>M87+7</f>
@@ -3491,12 +3705,14 @@
     <row r="89" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B89" s="1"/>
       <c r="H89" s="5">
-        <f>H88+7</f>
-        <v>46650</v>
-      </c>
-      <c r="J89" s="5">
-        <f t="shared" si="13"/>
-        <v>46656</v>
+        <f t="shared" ref="H89:H103" si="15">H88+7</f>
+        <v>46657</v>
+      </c>
+      <c r="J89" s="4">
+        <v>46041</v>
+      </c>
+      <c r="K89" s="4">
+        <v>45123</v>
       </c>
       <c r="M89" s="5">
         <f t="shared" ref="M89:M103" si="16">M88+7</f>
@@ -3506,12 +3722,12 @@
     <row r="90" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B90" s="1"/>
       <c r="H90" s="5">
-        <f t="shared" ref="H90:H104" si="17">H89+7</f>
-        <v>46657</v>
+        <f t="shared" si="15"/>
+        <v>46664</v>
       </c>
       <c r="J90" s="5">
-        <f t="shared" si="13"/>
-        <v>46663</v>
+        <f t="shared" ref="J90:J123" si="17">H70-1</f>
+        <v>46278</v>
       </c>
       <c r="M90" s="5">
         <f t="shared" si="16"/>
@@ -3521,12 +3737,12 @@
     <row r="91" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B91" s="1"/>
       <c r="H91" s="5">
+        <f t="shared" si="15"/>
+        <v>46671</v>
+      </c>
+      <c r="J91" s="5">
         <f t="shared" si="17"/>
-        <v>46664</v>
-      </c>
-      <c r="J91" s="5">
-        <f t="shared" si="13"/>
-        <v>46670</v>
+        <v>46285</v>
       </c>
       <c r="M91" s="5">
         <f t="shared" si="16"/>
@@ -3536,12 +3752,12 @@
     <row r="92" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B92" s="1"/>
       <c r="H92" s="5">
+        <f t="shared" si="15"/>
+        <v>46678</v>
+      </c>
+      <c r="J92" s="5">
         <f t="shared" si="17"/>
-        <v>46671</v>
-      </c>
-      <c r="J92" s="5">
-        <f t="shared" si="13"/>
-        <v>46677</v>
+        <v>46292</v>
       </c>
       <c r="M92" s="5">
         <f t="shared" si="16"/>
@@ -3551,12 +3767,12 @@
     <row r="93" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B93" s="1"/>
       <c r="H93" s="5">
+        <f t="shared" si="15"/>
+        <v>46685</v>
+      </c>
+      <c r="J93" s="5">
         <f t="shared" si="17"/>
-        <v>46678</v>
-      </c>
-      <c r="J93" s="5">
-        <f t="shared" si="13"/>
-        <v>46684</v>
+        <v>46299</v>
       </c>
       <c r="M93" s="5">
         <f t="shared" si="16"/>
@@ -3566,12 +3782,12 @@
     <row r="94" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B94" s="1"/>
       <c r="H94" s="5">
+        <f t="shared" si="15"/>
+        <v>46692</v>
+      </c>
+      <c r="J94" s="5">
         <f t="shared" si="17"/>
-        <v>46685</v>
-      </c>
-      <c r="J94" s="5">
-        <f t="shared" si="13"/>
-        <v>46691</v>
+        <v>46306</v>
       </c>
       <c r="M94" s="5">
         <f t="shared" si="16"/>
@@ -3581,12 +3797,12 @@
     <row r="95" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B95" s="1"/>
       <c r="H95" s="5">
+        <f t="shared" si="15"/>
+        <v>46699</v>
+      </c>
+      <c r="J95" s="5">
         <f t="shared" si="17"/>
-        <v>46692</v>
-      </c>
-      <c r="J95" s="5">
-        <f t="shared" si="13"/>
-        <v>46698</v>
+        <v>46313</v>
       </c>
       <c r="M95" s="5">
         <f t="shared" si="16"/>
@@ -3596,12 +3812,12 @@
     <row r="96" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B96" s="1"/>
       <c r="H96" s="5">
+        <f t="shared" si="15"/>
+        <v>46706</v>
+      </c>
+      <c r="J96" s="5">
         <f t="shared" si="17"/>
-        <v>46699</v>
-      </c>
-      <c r="J96" s="5">
-        <f t="shared" si="13"/>
-        <v>46705</v>
+        <v>46320</v>
       </c>
       <c r="M96" s="5">
         <f t="shared" si="16"/>
@@ -3611,12 +3827,12 @@
     <row r="97" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B97" s="1"/>
       <c r="H97" s="5">
+        <f t="shared" si="15"/>
+        <v>46713</v>
+      </c>
+      <c r="J97" s="5">
         <f t="shared" si="17"/>
-        <v>46706</v>
-      </c>
-      <c r="J97" s="5">
-        <f t="shared" si="13"/>
-        <v>46712</v>
+        <v>46327</v>
       </c>
       <c r="M97" s="5">
         <f t="shared" si="16"/>
@@ -3626,12 +3842,12 @@
     <row r="98" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B98" s="1"/>
       <c r="H98" s="5">
+        <f t="shared" si="15"/>
+        <v>46720</v>
+      </c>
+      <c r="J98" s="5">
         <f t="shared" si="17"/>
-        <v>46713</v>
-      </c>
-      <c r="J98" s="5">
-        <f t="shared" si="13"/>
-        <v>46719</v>
+        <v>46334</v>
       </c>
       <c r="M98" s="5">
         <f t="shared" si="16"/>
@@ -3641,12 +3857,12 @@
     <row r="99" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B99" s="1"/>
       <c r="H99" s="5">
+        <f t="shared" si="15"/>
+        <v>46727</v>
+      </c>
+      <c r="J99" s="5">
         <f t="shared" si="17"/>
-        <v>46720</v>
-      </c>
-      <c r="J99" s="5">
-        <f t="shared" si="13"/>
-        <v>46726</v>
+        <v>46341</v>
       </c>
       <c r="M99" s="5">
         <f t="shared" si="16"/>
@@ -3656,12 +3872,12 @@
     <row r="100" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B100" s="1"/>
       <c r="H100" s="5">
+        <f t="shared" si="15"/>
+        <v>46734</v>
+      </c>
+      <c r="J100" s="5">
         <f t="shared" si="17"/>
-        <v>46727</v>
-      </c>
-      <c r="J100" s="5">
-        <f t="shared" si="13"/>
-        <v>46733</v>
+        <v>46348</v>
       </c>
       <c r="M100" s="5">
         <f t="shared" si="16"/>
@@ -3671,12 +3887,12 @@
     <row r="101" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B101" s="1"/>
       <c r="H101" s="5">
+        <f t="shared" si="15"/>
+        <v>46741</v>
+      </c>
+      <c r="J101" s="5">
         <f t="shared" si="17"/>
-        <v>46734</v>
-      </c>
-      <c r="J101" s="5">
-        <f t="shared" si="13"/>
-        <v>46740</v>
+        <v>46355</v>
       </c>
       <c r="M101" s="5">
         <f t="shared" si="16"/>
@@ -3686,12 +3902,12 @@
     <row r="102" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B102" s="1"/>
       <c r="H102" s="5">
+        <f>H101+7</f>
+        <v>46748</v>
+      </c>
+      <c r="J102" s="5">
         <f t="shared" si="17"/>
-        <v>46741</v>
-      </c>
-      <c r="J102" s="5">
-        <f t="shared" si="13"/>
-        <v>46747</v>
+        <v>46362</v>
       </c>
       <c r="M102" s="5">
         <f t="shared" si="16"/>
@@ -3701,12 +3917,12 @@
     <row r="103" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B103" s="1"/>
       <c r="H103" s="5">
-        <f>H102+7</f>
-        <v>46748</v>
+        <f t="shared" si="15"/>
+        <v>46755</v>
       </c>
       <c r="J103" s="5">
-        <f t="shared" si="13"/>
-        <v>46754</v>
+        <f t="shared" si="17"/>
+        <v>46369</v>
       </c>
       <c r="M103" s="5">
         <f t="shared" si="16"/>
@@ -3715,82 +3931,158 @@
     </row>
     <row r="104" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B104" s="1"/>
-      <c r="H104" s="5">
+      <c r="J104" s="5">
         <f t="shared" si="17"/>
-        <v>46755</v>
+        <v>46376</v>
       </c>
     </row>
     <row r="105" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B105" s="1"/>
       <c r="H105" s="1"/>
+      <c r="J105" s="5">
+        <f t="shared" si="17"/>
+        <v>46383</v>
+      </c>
     </row>
     <row r="106" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B106" s="1"/>
+      <c r="J106" s="5">
+        <f t="shared" si="17"/>
+        <v>46390</v>
+      </c>
     </row>
     <row r="107" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B107" s="1"/>
+      <c r="J107" s="5">
+        <f t="shared" si="17"/>
+        <v>46642</v>
+      </c>
     </row>
     <row r="108" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B108" s="1"/>
+      <c r="J108" s="5">
+        <f t="shared" si="17"/>
+        <v>46649</v>
+      </c>
     </row>
     <row r="109" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B109" s="1"/>
+      <c r="J109" s="5">
+        <f t="shared" si="17"/>
+        <v>46656</v>
+      </c>
     </row>
     <row r="110" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B110" s="1"/>
+      <c r="J110" s="5">
+        <f t="shared" si="17"/>
+        <v>46663</v>
+      </c>
     </row>
     <row r="111" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B111" s="1"/>
+      <c r="J111" s="5">
+        <f t="shared" si="17"/>
+        <v>46670</v>
+      </c>
     </row>
     <row r="112" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B112" s="1"/>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J112" s="5">
+        <f t="shared" si="17"/>
+        <v>46677</v>
+      </c>
+    </row>
+    <row r="113" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B113" s="1"/>
-    </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J113" s="5">
+        <f t="shared" si="17"/>
+        <v>46684</v>
+      </c>
+    </row>
+    <row r="114" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B114" s="1"/>
-    </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J114" s="5">
+        <f t="shared" si="17"/>
+        <v>46691</v>
+      </c>
+    </row>
+    <row r="115" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B115" s="1"/>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J115" s="5">
+        <f t="shared" si="17"/>
+        <v>46698</v>
+      </c>
+    </row>
+    <row r="116" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B116" s="1"/>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J116" s="5">
+        <f t="shared" si="17"/>
+        <v>46705</v>
+      </c>
+    </row>
+    <row r="117" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B117" s="1"/>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J117" s="5">
+        <f t="shared" si="17"/>
+        <v>46712</v>
+      </c>
+    </row>
+    <row r="118" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B118" s="1"/>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J118" s="5">
+        <f t="shared" si="17"/>
+        <v>46719</v>
+      </c>
+    </row>
+    <row r="119" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B119" s="1"/>
-    </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J119" s="5">
+        <f t="shared" si="17"/>
+        <v>46726</v>
+      </c>
+    </row>
+    <row r="120" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B120" s="1"/>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J120" s="5">
+        <f t="shared" si="17"/>
+        <v>46733</v>
+      </c>
+    </row>
+    <row r="121" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B121" s="1"/>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J121" s="5">
+        <f t="shared" si="17"/>
+        <v>46740</v>
+      </c>
+    </row>
+    <row r="122" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B122" s="1"/>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J122" s="5">
+        <f t="shared" si="17"/>
+        <v>46747</v>
+      </c>
+    </row>
+    <row r="123" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B123" s="1"/>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="J123" s="5">
+        <f t="shared" si="17"/>
+        <v>46754</v>
+      </c>
+    </row>
+    <row r="124" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B128" s="1"/>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.35">
@@ -3824,8 +4116,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C9A9C83-5585-4ACC-9F40-AAEA8DEF72C1}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
@@ -3904,24 +4200,64 @@
         <v>45460</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>2025</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>175</v>
+        <v>235</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>177</v>
+        <v>232</v>
       </c>
       <c r="F5" s="1">
         <v>45830</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F6" s="1">
+        <v>46186</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2">
+        <v>2027</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="F7" s="1">
+        <v>46558</v>
       </c>
     </row>
   </sheetData>
@@ -3931,10 +4267,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADF483CF-28E5-47CE-B16F-35B62BA3AB9C}">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -3971,8 +4307,26 @@
       <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M1" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q1" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="R1" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -4009,8 +4363,26 @@
       <c r="L2" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M2" s="17">
+        <v>1</v>
+      </c>
+      <c r="N2" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="P2" s="17">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R2" s="16" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -4047,8 +4419,26 @@
       <c r="L3" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M3" s="17">
+        <v>2</v>
+      </c>
+      <c r="N3" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="P3" s="17">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R3" s="16" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -4085,8 +4475,26 @@
       <c r="L4" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M4" s="17">
+        <v>3</v>
+      </c>
+      <c r="N4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="P4" s="17">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R4" s="16" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -4123,8 +4531,26 @@
       <c r="L5" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M5" s="17">
+        <v>4</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O5" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="P5" s="17">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R5" s="16" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -4161,8 +4587,26 @@
       <c r="L6" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M6" s="17">
+        <v>5</v>
+      </c>
+      <c r="N6" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="P6" s="17">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R6" s="16" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -4199,8 +4643,26 @@
       <c r="L7" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M7" s="17">
+        <v>6</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O7" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="P7" s="17">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R7" s="16" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -4237,8 +4699,26 @@
       <c r="L8" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M8" s="17">
+        <v>7</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O8" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="P8" s="17">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R8" s="16" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -4275,8 +4755,26 @@
       <c r="L9" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M9" s="17">
+        <v>8</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O9" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="P9" s="17">
+        <v>8</v>
+      </c>
+      <c r="Q9" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R9" s="16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -4313,8 +4811,26 @@
       <c r="L10" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M10" s="17">
+        <v>9</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O10" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="P10" s="17">
+        <v>9</v>
+      </c>
+      <c r="Q10" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R10" s="16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -4351,8 +4867,26 @@
       <c r="L11" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M11" s="17">
+        <v>10</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O11" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="P11" s="17">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R11" s="16" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -4389,8 +4923,26 @@
       <c r="L12" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M12" s="17">
+        <v>11</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O12" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="P12" s="17">
+        <v>11</v>
+      </c>
+      <c r="Q12" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R12" s="16" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -4427,8 +4979,26 @@
       <c r="L13" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M13" s="17">
+        <v>12</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O13" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="P13" s="17">
+        <v>12</v>
+      </c>
+      <c r="Q13" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R13" s="16" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -4465,8 +5035,26 @@
       <c r="L14" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M14" s="17">
+        <v>13</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O14" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="P14" s="17">
+        <v>13</v>
+      </c>
+      <c r="Q14" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R14" s="16" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -4503,8 +5091,26 @@
       <c r="L15" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M15" s="17">
+        <v>14</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O15" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="P15" s="17">
+        <v>14</v>
+      </c>
+      <c r="Q15" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R15" s="16" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -4541,8 +5147,26 @@
       <c r="L16" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M16" s="17">
+        <v>15</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="P16" s="17">
+        <v>15</v>
+      </c>
+      <c r="Q16" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R16" s="16" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -4579,8 +5203,26 @@
       <c r="L17" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M17" s="17">
+        <v>16</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O17" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="P17" s="17">
+        <v>16</v>
+      </c>
+      <c r="Q17" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R17" s="16" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -4617,9 +5259,28 @@
       <c r="L18" s="2" t="s">
         <v>79</v>
       </c>
+      <c r="M18" s="17">
+        <v>17</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O18" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="P18" s="17">
+        <v>17</v>
+      </c>
+      <c r="Q18" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R18" s="16" t="s">
+        <v>231</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4706,8 +5367,14 @@
       <c r="L2" s="1">
         <v>45904</v>
       </c>
+      <c r="M2" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="N2" s="1">
         <v>46275</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="P2" s="1">
         <v>46639</v>
@@ -4754,10 +5421,16 @@
         <f>L2+7</f>
         <v>45911</v>
       </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
       <c r="N3" s="1">
         <f>N2+7</f>
         <v>46282</v>
       </c>
+      <c r="O3">
+        <v>2</v>
+      </c>
       <c r="P3" s="1">
         <f>P2+7</f>
         <v>46646</v>
@@ -4804,10 +5477,16 @@
         <f t="shared" ref="L4:L18" si="3">L3+7</f>
         <v>45918</v>
       </c>
+      <c r="M4">
+        <v>3</v>
+      </c>
       <c r="N4" s="1">
         <f>N3+7</f>
         <v>46289</v>
       </c>
+      <c r="O4">
+        <v>3</v>
+      </c>
       <c r="P4" s="1">
         <f t="shared" ref="P4:P18" si="4">P3+7</f>
         <v>46653</v>
@@ -4854,10 +5533,16 @@
         <f t="shared" si="3"/>
         <v>45925</v>
       </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
       <c r="N5" s="1">
         <f t="shared" ref="N5:N18" si="5">N4+7</f>
         <v>46296</v>
       </c>
+      <c r="O5">
+        <v>4</v>
+      </c>
       <c r="P5" s="1">
         <f t="shared" si="4"/>
         <v>46660</v>
@@ -4904,10 +5589,16 @@
         <f t="shared" si="3"/>
         <v>45932</v>
       </c>
+      <c r="M6">
+        <v>5</v>
+      </c>
       <c r="N6" s="1">
         <f t="shared" si="5"/>
         <v>46303</v>
       </c>
+      <c r="O6">
+        <v>5</v>
+      </c>
       <c r="P6" s="1">
         <f t="shared" si="4"/>
         <v>46667</v>
@@ -4954,10 +5645,16 @@
         <f t="shared" si="3"/>
         <v>45939</v>
       </c>
+      <c r="M7">
+        <v>6</v>
+      </c>
       <c r="N7" s="1">
         <f t="shared" si="5"/>
         <v>46310</v>
       </c>
+      <c r="O7">
+        <v>6</v>
+      </c>
       <c r="P7" s="1">
         <f t="shared" si="4"/>
         <v>46674</v>
@@ -5004,10 +5701,16 @@
         <f t="shared" si="3"/>
         <v>45946</v>
       </c>
+      <c r="M8">
+        <v>7</v>
+      </c>
       <c r="N8" s="1">
         <f t="shared" si="5"/>
         <v>46317</v>
       </c>
+      <c r="O8">
+        <v>7</v>
+      </c>
       <c r="P8" s="1">
         <f t="shared" si="4"/>
         <v>46681</v>
@@ -5054,10 +5757,16 @@
         <f t="shared" si="3"/>
         <v>45953</v>
       </c>
+      <c r="M9">
+        <v>8</v>
+      </c>
       <c r="N9" s="1">
         <f t="shared" si="5"/>
         <v>46324</v>
       </c>
+      <c r="O9">
+        <v>8</v>
+      </c>
       <c r="P9" s="1">
         <f t="shared" si="4"/>
         <v>46688</v>
@@ -5104,10 +5813,16 @@
         <f t="shared" si="3"/>
         <v>45960</v>
       </c>
+      <c r="M10">
+        <v>9</v>
+      </c>
       <c r="N10" s="1">
         <f t="shared" si="5"/>
         <v>46331</v>
       </c>
+      <c r="O10">
+        <v>9</v>
+      </c>
       <c r="P10" s="1">
         <f t="shared" si="4"/>
         <v>46695</v>
@@ -5154,10 +5869,16 @@
         <f t="shared" si="3"/>
         <v>45967</v>
       </c>
+      <c r="M11">
+        <v>10</v>
+      </c>
       <c r="N11" s="1">
         <f t="shared" si="5"/>
         <v>46338</v>
       </c>
+      <c r="O11">
+        <v>10</v>
+      </c>
       <c r="P11" s="1">
         <f t="shared" si="4"/>
         <v>46702</v>
@@ -5204,10 +5925,16 @@
         <f t="shared" si="3"/>
         <v>45974</v>
       </c>
+      <c r="M12">
+        <v>11</v>
+      </c>
       <c r="N12" s="1">
         <f t="shared" si="5"/>
         <v>46345</v>
       </c>
+      <c r="O12">
+        <v>11</v>
+      </c>
       <c r="P12" s="1">
         <f t="shared" si="4"/>
         <v>46709</v>
@@ -5254,10 +5981,16 @@
         <f t="shared" si="3"/>
         <v>45981</v>
       </c>
+      <c r="M13" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="N13" s="1">
         <f t="shared" si="5"/>
         <v>46352</v>
       </c>
+      <c r="O13" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="P13" s="1">
         <f t="shared" si="4"/>
         <v>46716</v>
@@ -5304,10 +6037,16 @@
         <f t="shared" si="3"/>
         <v>45988</v>
       </c>
+      <c r="M14">
+        <v>13</v>
+      </c>
       <c r="N14" s="1">
         <f t="shared" si="5"/>
         <v>46359</v>
       </c>
+      <c r="O14">
+        <v>13</v>
+      </c>
       <c r="P14" s="1">
         <f t="shared" si="4"/>
         <v>46723</v>
@@ -5354,10 +6093,16 @@
         <f t="shared" si="3"/>
         <v>45995</v>
       </c>
+      <c r="M15">
+        <v>14</v>
+      </c>
       <c r="N15" s="1">
         <f t="shared" si="5"/>
         <v>46366</v>
       </c>
+      <c r="O15">
+        <v>14</v>
+      </c>
       <c r="P15" s="1">
         <f t="shared" si="4"/>
         <v>46730</v>
@@ -5404,10 +6149,16 @@
         <f t="shared" si="3"/>
         <v>46002</v>
       </c>
+      <c r="M16">
+        <v>15</v>
+      </c>
       <c r="N16" s="1">
         <f t="shared" si="5"/>
         <v>46373</v>
       </c>
+      <c r="O16">
+        <v>15</v>
+      </c>
       <c r="P16" s="1">
         <f t="shared" si="4"/>
         <v>46737</v>
@@ -5454,10 +6205,16 @@
         <f t="shared" si="3"/>
         <v>46009</v>
       </c>
+      <c r="M17">
+        <v>16</v>
+      </c>
       <c r="N17" s="1">
         <f t="shared" si="5"/>
         <v>46380</v>
       </c>
+      <c r="O17">
+        <v>16</v>
+      </c>
       <c r="P17" s="1">
         <f t="shared" si="4"/>
         <v>46744</v>
@@ -5504,9 +6261,15 @@
         <f t="shared" si="3"/>
         <v>46016</v>
       </c>
+      <c r="M18">
+        <v>17</v>
+      </c>
       <c r="N18" s="1">
         <f t="shared" si="5"/>
         <v>46387</v>
+      </c>
+      <c r="O18">
+        <v>17</v>
       </c>
       <c r="P18" s="1">
         <f t="shared" si="4"/>
@@ -5532,10 +6295,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -5561,7 +6324,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C4" s="9"/>
     </row>
@@ -5570,7 +6333,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C5" s="9"/>
     </row>
@@ -5579,7 +6342,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C6" s="9"/>
     </row>
@@ -5588,7 +6351,7 @@
         <v>62</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C7" s="9"/>
     </row>
@@ -5597,7 +6360,7 @@
         <v>80</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C8" s="9"/>
     </row>
@@ -5606,7 +6369,7 @@
         <v>82</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C9" s="9"/>
     </row>
@@ -5615,16 +6378,16 @@
         <v>83</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C10" s="9"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C11" s="9"/>
     </row>
@@ -5633,36 +6396,36 @@
         <v>84</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C12" s="9"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C13" s="9"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C14" s="9"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>